<commit_message>
Actualización automática: 2026-06-05 18:14:05
</commit_message>
<xml_diff>
--- a/Zabbix_agent/Salidas_Playbooks/zbx_monitores_top5.xlsx
+++ b/Zabbix_agent/Salidas_Playbooks/zbx_monitores_top5.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>InventoryHostname</t>
   </si>
@@ -37,10 +37,13 @@
     <t>Monitores_Creados</t>
   </si>
   <si>
-    <t>mongo-prd-n2</t>
-  </si>
-  <si>
-    <t>10.181.34.4</t>
+    <t>vm-eu2-appdru04-prd</t>
+  </si>
+  <si>
+    <t>VM-EU2-APPDRU04-PRD</t>
+  </si>
+  <si>
+    <t>10.0.16.109</t>
   </si>
   <si>
     <t>aplicado</t>
@@ -49,7 +52,7 @@
     <t>active</t>
   </si>
   <si>
-    <t>zabbix_agent2 (Zabbix) 7.0.10</t>
+    <t>zabbix_agent2 (Zabbix) 7.0.18</t>
   </si>
   <si>
     <t>si</t>
@@ -433,22 +436,22 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática: 2026-06-19 12:12:52
</commit_message>
<xml_diff>
--- a/Zabbix_agent/Salidas_Playbooks/zbx_monitores_top5.xlsx
+++ b/Zabbix_agent/Salidas_Playbooks/zbx_monitores_top5.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="37">
   <si>
     <t>InventoryHostname</t>
   </si>
@@ -37,6 +37,60 @@
     <t>Monitores_Creados</t>
   </si>
   <si>
+    <t>vm-eu2-appdru03-rst</t>
+  </si>
+  <si>
+    <t>VM-EU2-APPDRU03-RST</t>
+  </si>
+  <si>
+    <t>10.0.16.149</t>
+  </si>
+  <si>
+    <t>no-aplico</t>
+  </si>
+  <si>
+    <t>active</t>
+  </si>
+  <si>
+    <t>zabbix_agent2 (Zabbix) 7.0.18</t>
+  </si>
+  <si>
+    <t>ya_existian</t>
+  </si>
+  <si>
+    <t>vm-eu2-appdru04-prd</t>
+  </si>
+  <si>
+    <t>VM-EU2-APPDRU04-PRD</t>
+  </si>
+  <si>
+    <t>10.0.16.109</t>
+  </si>
+  <si>
+    <t>vm-eu2-dbdru02-prd</t>
+  </si>
+  <si>
+    <t>VM-EU2-DBDRU02-PRD</t>
+  </si>
+  <si>
+    <t>10.0.16.157</t>
+  </si>
+  <si>
+    <t>aplicado</t>
+  </si>
+  <si>
+    <t>si</t>
+  </si>
+  <si>
+    <t>vm-eu2-dbdru03-prd</t>
+  </si>
+  <si>
+    <t>VM-EU2-DBDRU03-PRD</t>
+  </si>
+  <si>
+    <t>10.0.16.158</t>
+  </si>
+  <si>
     <t>vm-eu2-devopscomp-prd</t>
   </si>
   <si>
@@ -46,16 +100,31 @@
     <t>10.0.16.61</t>
   </si>
   <si>
-    <t>aplicado</t>
-  </si>
-  <si>
-    <t>active</t>
-  </si>
-  <si>
-    <t>zabbix_agent2 (Zabbix) 7.0.18</t>
-  </si>
-  <si>
-    <t>si</t>
+    <t>vm-eu2-zic3-prd</t>
+  </si>
+  <si>
+    <t>VM-EU2-SROUT-PRD</t>
+  </si>
+  <si>
+    <t>10.0.31.5</t>
+  </si>
+  <si>
+    <t>vm-eu2-srout-prd</t>
+  </si>
+  <si>
+    <t>vm-eu2-sic3-prd</t>
+  </si>
+  <si>
+    <t>10.0.16.132</t>
+  </si>
+  <si>
+    <t>vm-eu2-tdp-prd</t>
+  </si>
+  <si>
+    <t>VM-EU2-TDP-PRD</t>
+  </si>
+  <si>
+    <t>10.0.16.133</t>
   </si>
 </sst>
 </file>
@@ -402,7 +471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="7" width="22.7109375" customWidth="1"/>
@@ -454,6 +523,167 @@
         <v>13</v>
       </c>
     </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>